<commit_message>
updated crit_data.xlsx and topicsCourseCatalog.js
</commit_message>
<xml_diff>
--- a/cirt_data.xlsx
+++ b/cirt_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://o365coloradoedu-my.sharepoint.com/personal/daad2295_colorado_edu/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="173" documentId="8_{9DEE3B3B-C278-45E7-AFEB-FC7D865F8C7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F94D6800-BE81-42EB-8111-3F4D9F2E7C98}"/>
+  <xr:revisionPtr revIDLastSave="198" documentId="8_{9DEE3B3B-C278-45E7-AFEB-FC7D865F8C7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{615EC137-2975-4E2A-B918-6E1966ADF36F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{969D6A76-162A-4286-A653-6BBA36AECB0D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{969D6A76-162A-4286-A653-6BBA36AECB0D}"/>
   </bookViews>
   <sheets>
     <sheet name="courses" sheetId="1" r:id="rId1"/>
@@ -8878,6 +8878,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -35183,7 +35187,8 @@
   <dimension ref="A1:U604"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="9.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" customWidth="1"/>
     <col min="3" max="3" width="14.140625" customWidth="1"/>
     <col min="4" max="4" width="9.85546875" style="3" customWidth="1"/>
     <col min="5" max="5" width="31.42578125" customWidth="1"/>
@@ -35310,19 +35315,19 @@
         <v>2323</v>
       </c>
       <c r="Q2" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R2" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S2" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T2" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U2" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
@@ -35378,16 +35383,16 @@
         <v>50</v>
       </c>
       <c r="R3" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S3" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T3" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U3" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U3" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
@@ -35440,19 +35445,19 @@
         <v>2335</v>
       </c>
       <c r="Q4" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R4" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S4" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T4" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U4" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U4" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
@@ -35505,19 +35510,19 @@
         <v>2323</v>
       </c>
       <c r="Q5" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R5" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S5" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T5" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U5" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U5" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
@@ -35570,19 +35575,19 @@
         <v>2323</v>
       </c>
       <c r="Q6" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R6" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S6" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T6" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U6" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U6" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="7" spans="1:21" ht="15.75" x14ac:dyDescent="0.3">
@@ -35638,16 +35643,16 @@
         <v>59</v>
       </c>
       <c r="R7" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S7" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T7" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U7" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
@@ -35700,19 +35705,19 @@
         <v>2323</v>
       </c>
       <c r="Q8" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R8" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S8" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T8" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U8" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U8" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
@@ -35765,19 +35770,19 @@
         <v>2323</v>
       </c>
       <c r="Q9" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R9" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S9" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T9" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U9" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U9" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
@@ -35830,19 +35835,19 @@
         <v>2323</v>
       </c>
       <c r="Q10" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R10" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S10" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T10" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U10" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U10" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
@@ -35895,19 +35900,19 @@
         <v>2323</v>
       </c>
       <c r="Q11" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R11" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S11" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T11" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U11" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U11" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
@@ -35960,19 +35965,19 @@
         <v>2323</v>
       </c>
       <c r="Q12" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R12" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S12" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T12" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U12" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U12" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
@@ -36025,19 +36030,19 @@
         <v>2323</v>
       </c>
       <c r="Q13" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R13" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S13" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T13" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U13" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U13" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
@@ -36090,19 +36095,19 @@
         <v>2323</v>
       </c>
       <c r="Q14" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R14" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S14" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T14" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U14" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U14" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
@@ -36158,16 +36163,16 @@
         <v>77</v>
       </c>
       <c r="R15" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S15" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T15" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U15" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U15" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
@@ -36220,19 +36225,19 @@
         <v>2323</v>
       </c>
       <c r="Q16" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R16" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S16" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T16" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U16" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U16" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
@@ -36285,19 +36290,19 @@
         <v>2323</v>
       </c>
       <c r="Q17" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R17" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S17" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T17" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U17" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U17" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
@@ -36350,19 +36355,19 @@
         <v>2323</v>
       </c>
       <c r="Q18" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R18" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S18" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T18" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U18" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U18" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
@@ -36415,19 +36420,19 @@
         <v>2335</v>
       </c>
       <c r="Q19" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R19" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S19" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T19" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U19" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U19" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
@@ -36480,19 +36485,19 @@
         <v>2335</v>
       </c>
       <c r="Q20" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R20" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S20" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T20" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U20" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U20" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
@@ -36545,19 +36550,19 @@
         <v>2335</v>
       </c>
       <c r="Q21" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R21" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S21" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T21" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U21" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U21" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
@@ -36610,19 +36615,19 @@
         <v>2335</v>
       </c>
       <c r="Q22" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R22" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S22" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T22" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U22" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U22" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
@@ -36675,19 +36680,19 @@
         <v>2349</v>
       </c>
       <c r="Q23" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R23" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S23" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T23" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U23" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U23" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
@@ -36740,19 +36745,19 @@
         <v>2323</v>
       </c>
       <c r="Q24" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R24" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S24" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T24" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U24" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U24" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
@@ -36808,16 +36813,16 @@
         <v>59</v>
       </c>
       <c r="R25" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S25" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T25" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U25" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U25" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
@@ -36870,19 +36875,19 @@
         <v>2323</v>
       </c>
       <c r="Q26" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R26" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S26" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T26" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U26" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U26" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
@@ -36935,19 +36940,19 @@
         <v>2323</v>
       </c>
       <c r="Q27" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R27" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S27" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T27" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U27" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U27" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
@@ -37000,19 +37005,19 @@
         <v>2323</v>
       </c>
       <c r="Q28" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R28" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S28" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T28" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U28" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U28" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -37068,16 +37073,16 @@
         <v>59</v>
       </c>
       <c r="R29" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S29" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T29" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U29" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U29" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -37130,19 +37135,19 @@
         <v>2323</v>
       </c>
       <c r="Q30" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R30" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S30" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T30" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U30" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U30" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -37195,19 +37200,19 @@
         <v>2323</v>
       </c>
       <c r="Q31" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R31" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S31" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T31" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U31" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U31" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -37260,19 +37265,19 @@
         <v>2335</v>
       </c>
       <c r="Q32" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R32" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S32" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T32" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U32" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U32" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
@@ -37325,19 +37330,19 @@
         <v>2335</v>
       </c>
       <c r="Q33" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R33" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S33" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T33" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U33" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U33" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
@@ -37390,19 +37395,19 @@
         <v>2335</v>
       </c>
       <c r="Q34" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R34" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S34" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T34" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U34" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U34" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
@@ -37455,19 +37460,19 @@
         <v>2335</v>
       </c>
       <c r="Q35" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R35" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S35" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T35" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U35" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U35" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
@@ -37520,19 +37525,19 @@
         <v>2335</v>
       </c>
       <c r="Q36" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R36" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S36" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T36" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U36" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U36" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
@@ -37588,16 +37593,16 @@
         <v>59</v>
       </c>
       <c r="R37" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S37" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T37" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U37" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U37" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
@@ -37650,19 +37655,19 @@
         <v>2323</v>
       </c>
       <c r="Q38" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R38" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S38" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T38" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U38" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U38" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
@@ -37715,19 +37720,19 @@
         <v>2323</v>
       </c>
       <c r="Q39" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R39" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S39" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T39" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U39" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U39" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
@@ -37783,16 +37788,16 @@
         <v>130</v>
       </c>
       <c r="R40" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S40" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T40" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U40" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U40" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
@@ -37845,19 +37850,19 @@
         <v>2323</v>
       </c>
       <c r="Q41" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R41" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S41" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T41" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U41" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U41" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
@@ -37910,19 +37915,19 @@
         <v>2335</v>
       </c>
       <c r="Q42" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R42" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S42" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T42" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U42" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U42" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
@@ -37978,16 +37983,16 @@
         <v>130</v>
       </c>
       <c r="R43" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S43" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T43" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U43" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U43" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
@@ -38040,19 +38045,19 @@
         <v>2323</v>
       </c>
       <c r="Q44" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R44" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S44" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T44" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U44" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U44" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
@@ -38105,19 +38110,19 @@
         <v>2335</v>
       </c>
       <c r="Q45" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R45" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S45" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T45" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U45" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U45" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
@@ -38173,16 +38178,16 @@
         <v>130</v>
       </c>
       <c r="R46" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S46" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T46" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U46" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U46" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
@@ -38235,19 +38240,19 @@
         <v>2335</v>
       </c>
       <c r="Q47" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R47" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S47" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T47" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U47" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U47" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
@@ -38300,19 +38305,19 @@
         <v>2323</v>
       </c>
       <c r="Q48" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R48" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S48" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T48" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U48" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U48" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
@@ -38365,19 +38370,19 @@
         <v>2349</v>
       </c>
       <c r="Q49" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R49" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S49" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T49" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U49" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U49" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
@@ -38430,19 +38435,19 @@
         <v>2335</v>
       </c>
       <c r="Q50" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R50" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S50" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T50" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U50" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U50" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -38495,19 +38500,19 @@
         <v>2323</v>
       </c>
       <c r="Q51" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R51" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S51" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T51" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U51" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U51" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
@@ -38560,19 +38565,19 @@
         <v>2323</v>
       </c>
       <c r="Q52" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R52" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S52" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T52" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U52" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U52" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
@@ -38625,19 +38630,19 @@
         <v>2323</v>
       </c>
       <c r="Q53" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R53" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S53" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T53" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U53" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U53" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
@@ -38690,19 +38695,19 @@
         <v>2335</v>
       </c>
       <c r="Q54" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R54" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S54" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T54" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U54" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U54" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
@@ -38758,16 +38763,16 @@
         <v>59</v>
       </c>
       <c r="R55" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S55" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T55" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U55" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U55" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
@@ -38820,19 +38825,19 @@
         <v>2323</v>
       </c>
       <c r="Q56" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R56" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S56" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T56" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U56" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U56" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -38888,16 +38893,16 @@
         <v>59</v>
       </c>
       <c r="R57" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S57" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T57" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U57" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U57" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
@@ -38950,19 +38955,19 @@
         <v>2323</v>
       </c>
       <c r="Q58" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R58" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S58" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T58" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U58" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U58" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
@@ -39015,19 +39020,19 @@
         <v>2323</v>
       </c>
       <c r="Q59" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R59" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S59" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T59" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U59" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U59" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -39080,19 +39085,19 @@
         <v>2323</v>
       </c>
       <c r="Q60" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R60" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S60" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T60" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U60" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U60" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -39145,19 +39150,19 @@
         <v>2350</v>
       </c>
       <c r="Q61" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R61" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S61" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T61" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U61" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U61" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -39210,19 +39215,19 @@
         <v>2350</v>
       </c>
       <c r="Q62" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R62" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S62" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T62" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U62" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U62" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
@@ -39275,7 +39280,7 @@
         <v>2348</v>
       </c>
       <c r="Q63" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R63" t="s">
         <v>2643</v>
@@ -39286,8 +39291,8 @@
       <c r="T63" t="s">
         <v>2641</v>
       </c>
-      <c r="U63" s="1" t="s">
-        <v>2493</v>
+      <c r="U63" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
@@ -39340,19 +39345,19 @@
         <v>2323</v>
       </c>
       <c r="Q64" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R64" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S64" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T64" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U64" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U64" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
@@ -39405,19 +39410,19 @@
         <v>2323</v>
       </c>
       <c r="Q65" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R65" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S65" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T65" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U65" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U65" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
@@ -39470,19 +39475,19 @@
         <v>2323</v>
       </c>
       <c r="Q66" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R66" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S66" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T66" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U66" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U66" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
@@ -39538,16 +39543,16 @@
         <v>2545</v>
       </c>
       <c r="R67" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S67" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T67" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U67" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U67" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -39603,16 +39608,16 @@
         <v>2544</v>
       </c>
       <c r="R68" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S68" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T68" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U68" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U68" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
@@ -39665,19 +39670,19 @@
         <v>2323</v>
       </c>
       <c r="Q69" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R69" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S69" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T69" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U69" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U69" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
@@ -39730,19 +39735,19 @@
         <v>2335</v>
       </c>
       <c r="Q70" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R70" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S70" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T70" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U70" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U70" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
@@ -39795,19 +39800,19 @@
         <v>2323</v>
       </c>
       <c r="Q71" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R71" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S71" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T71" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U71" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U71" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
@@ -39860,19 +39865,19 @@
         <v>2350</v>
       </c>
       <c r="Q72" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R72" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S72" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T72" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U72" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U72" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
@@ -39925,7 +39930,7 @@
         <v>2323</v>
       </c>
       <c r="Q73" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R73" t="s">
         <v>2643</v>
@@ -39936,8 +39941,8 @@
       <c r="T73" t="s">
         <v>2641</v>
       </c>
-      <c r="U73" s="1" t="s">
-        <v>2493</v>
+      <c r="U73" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -39993,16 +39998,16 @@
         <v>2494</v>
       </c>
       <c r="R74" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S74" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T74" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U74" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U74" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
@@ -40055,19 +40060,19 @@
         <v>2323</v>
       </c>
       <c r="Q75" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R75" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S75" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T75" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U75" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U75" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -40120,19 +40125,19 @@
         <v>2323</v>
       </c>
       <c r="Q76" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R76" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S76" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T76" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U76" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U76" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
@@ -40185,19 +40190,19 @@
         <v>2323</v>
       </c>
       <c r="Q77" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R77" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S77" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T77" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U77" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U77" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
@@ -40253,16 +40258,16 @@
         <v>2494</v>
       </c>
       <c r="R78" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S78" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T78" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U78" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U78" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
@@ -40315,19 +40320,19 @@
         <v>2323</v>
       </c>
       <c r="Q79" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R79" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S79" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T79" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U79" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U79" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
@@ -40380,19 +40385,19 @@
         <v>2323</v>
       </c>
       <c r="Q80" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R80" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S80" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T80" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U80" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U80" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
@@ -40445,19 +40450,19 @@
         <v>2323</v>
       </c>
       <c r="Q81" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R81" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S81" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T81" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U81" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U81" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
@@ -40510,19 +40515,19 @@
         <v>2323</v>
       </c>
       <c r="Q82" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R82" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S82" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T82" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U82" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U82" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
@@ -40575,19 +40580,19 @@
         <v>2323</v>
       </c>
       <c r="Q83" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R83" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S83" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T83" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U83" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U83" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
@@ -40640,19 +40645,19 @@
         <v>2323</v>
       </c>
       <c r="Q84" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R84" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S84" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T84" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U84" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U84" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
@@ -40705,19 +40710,19 @@
         <v>2335</v>
       </c>
       <c r="Q85" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R85" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S85" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T85" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U85" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U85" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
@@ -40770,7 +40775,7 @@
         <v>2323</v>
       </c>
       <c r="Q86" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R86" t="s">
         <v>2643</v>
@@ -40781,8 +40786,8 @@
       <c r="T86" t="s">
         <v>2641</v>
       </c>
-      <c r="U86" s="1" t="s">
-        <v>2493</v>
+      <c r="U86" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
@@ -40838,16 +40843,16 @@
         <v>2544</v>
       </c>
       <c r="R87" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S87" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T87" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U87" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U87" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
@@ -40900,19 +40905,19 @@
         <v>2323</v>
       </c>
       <c r="Q88" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R88" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S88" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T88" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U88" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U88" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
@@ -40965,19 +40970,19 @@
         <v>2323</v>
       </c>
       <c r="Q89" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R89" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S89" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T89" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U89" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U89" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
@@ -41030,19 +41035,19 @@
         <v>2350</v>
       </c>
       <c r="Q90" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R90" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S90" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T90" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U90" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U90" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
@@ -41095,19 +41100,19 @@
         <v>2323</v>
       </c>
       <c r="Q91" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R91" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S91" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T91" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U91" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U91" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
@@ -41160,19 +41165,19 @@
         <v>2351</v>
       </c>
       <c r="Q92" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R92" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S92" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T92" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U92" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U92" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
@@ -41225,19 +41230,19 @@
         <v>2351</v>
       </c>
       <c r="Q93" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R93" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S93" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T93" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U93" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U93" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
@@ -41293,16 +41298,16 @@
         <v>2535</v>
       </c>
       <c r="R94" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S94" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T94" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U94" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U94" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
@@ -41355,19 +41360,19 @@
         <v>2323</v>
       </c>
       <c r="Q95" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R95" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S95" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T95" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U95" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U95" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
@@ -41420,19 +41425,19 @@
         <v>2323</v>
       </c>
       <c r="Q96" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R96" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S96" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T96" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U96" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U96" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
@@ -41485,19 +41490,19 @@
         <v>2323</v>
       </c>
       <c r="Q97" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R97" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S97" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T97" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U97" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U97" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
@@ -41550,19 +41555,19 @@
         <v>2323</v>
       </c>
       <c r="Q98" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R98" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S98" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T98" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U98" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U98" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
@@ -41615,19 +41620,19 @@
         <v>2323</v>
       </c>
       <c r="Q99" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R99" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S99" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T99" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U99" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U99" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
@@ -41683,16 +41688,16 @@
         <v>224</v>
       </c>
       <c r="R100" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S100" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T100" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U100" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U100" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.25">
@@ -41745,19 +41750,19 @@
         <v>2323</v>
       </c>
       <c r="Q101" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R101" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S101" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T101" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U101" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U101" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
@@ -41810,19 +41815,19 @@
         <v>2351</v>
       </c>
       <c r="Q102" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R102" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S102" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T102" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U102" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U102" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.25">
@@ -41875,19 +41880,19 @@
         <v>2335</v>
       </c>
       <c r="Q103" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R103" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S103" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T103" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U103" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U103" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.25">
@@ -41940,19 +41945,19 @@
         <v>2323</v>
       </c>
       <c r="Q104" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R104" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S104" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T104" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U104" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U104" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
@@ -42005,19 +42010,19 @@
         <v>2335</v>
       </c>
       <c r="Q105" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R105" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S105" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T105" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U105" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U105" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.25">
@@ -42073,16 +42078,16 @@
         <v>2494</v>
       </c>
       <c r="R106" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S106" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T106" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U106" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U106" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
@@ -42135,19 +42140,19 @@
         <v>2323</v>
       </c>
       <c r="Q107" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R107" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S107" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T107" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U107" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U107" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
@@ -42203,16 +42208,16 @@
         <v>2494</v>
       </c>
       <c r="R108" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S108" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T108" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U108" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U108" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
@@ -42265,19 +42270,19 @@
         <v>2323</v>
       </c>
       <c r="Q109" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R109" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S109" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T109" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U109" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U109" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
@@ -42330,19 +42335,19 @@
         <v>2323</v>
       </c>
       <c r="Q110" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R110" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S110" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T110" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U110" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U110" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
@@ -42395,19 +42400,19 @@
         <v>2323</v>
       </c>
       <c r="Q111" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R111" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S111" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T111" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U111" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U111" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="112" spans="1:21" x14ac:dyDescent="0.25">
@@ -42463,16 +42468,16 @@
         <v>2494</v>
       </c>
       <c r="R112" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S112" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T112" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U112" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U112" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
@@ -42525,19 +42530,19 @@
         <v>2323</v>
       </c>
       <c r="Q113" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R113" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S113" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T113" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U113" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U113" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.25">
@@ -42590,19 +42595,19 @@
         <v>2323</v>
       </c>
       <c r="Q114" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R114" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S114" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T114" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U114" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U114" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">
@@ -42655,19 +42660,19 @@
         <v>2323</v>
       </c>
       <c r="Q115" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R115" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S115" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T115" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U115" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U115" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.25">
@@ -42720,19 +42725,19 @@
         <v>2323</v>
       </c>
       <c r="Q116" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R116" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S116" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T116" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U116" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U116" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.25">
@@ -42785,19 +42790,19 @@
         <v>2323</v>
       </c>
       <c r="Q117" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R117" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S117" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T117" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U117" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U117" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="118" spans="1:21" x14ac:dyDescent="0.25">
@@ -42850,19 +42855,19 @@
         <v>2323</v>
       </c>
       <c r="Q118" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R118" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S118" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T118" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U118" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U118" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.25">
@@ -42915,19 +42920,19 @@
         <v>2335</v>
       </c>
       <c r="Q119" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R119" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S119" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T119" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U119" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U119" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="120" spans="1:21" x14ac:dyDescent="0.25">
@@ -42980,19 +42985,19 @@
         <v>2335</v>
       </c>
       <c r="Q120" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R120" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S120" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T120" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U120" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U120" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.25">
@@ -43045,19 +43050,19 @@
         <v>2323</v>
       </c>
       <c r="Q121" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R121" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S121" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T121" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U121" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U121" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="122" spans="1:21" x14ac:dyDescent="0.25">
@@ -43113,16 +43118,16 @@
         <v>2230</v>
       </c>
       <c r="R122" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S122" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T122" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U122" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U122" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="123" spans="1:21" x14ac:dyDescent="0.25">
@@ -43175,19 +43180,19 @@
         <v>2351</v>
       </c>
       <c r="Q123" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R123" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S123" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T123" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U123" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U123" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="124" spans="1:21" x14ac:dyDescent="0.25">
@@ -43240,19 +43245,19 @@
         <v>2323</v>
       </c>
       <c r="Q124" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R124" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S124" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T124" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U124" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U124" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="125" spans="1:21" x14ac:dyDescent="0.25">
@@ -43305,19 +43310,19 @@
         <v>2323</v>
       </c>
       <c r="Q125" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R125" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S125" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T125" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U125" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U125" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="126" spans="1:21" x14ac:dyDescent="0.25">
@@ -43370,19 +43375,19 @@
         <v>2323</v>
       </c>
       <c r="Q126" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R126" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S126" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T126" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U126" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U126" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="127" spans="1:21" x14ac:dyDescent="0.25">
@@ -43435,19 +43440,19 @@
         <v>2323</v>
       </c>
       <c r="Q127" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R127" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S127" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T127" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U127" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U127" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="128" spans="1:21" x14ac:dyDescent="0.25">
@@ -43500,19 +43505,19 @@
         <v>2323</v>
       </c>
       <c r="Q128" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R128" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S128" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T128" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U128" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U128" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="129" spans="1:21" x14ac:dyDescent="0.25">
@@ -43565,19 +43570,19 @@
         <v>2323</v>
       </c>
       <c r="Q129" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R129" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S129" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T129" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U129" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U129" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="130" spans="1:21" x14ac:dyDescent="0.25">
@@ -43630,19 +43635,19 @@
         <v>2350</v>
       </c>
       <c r="Q130" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R130" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S130" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T130" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U130" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U130" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
@@ -43695,19 +43700,19 @@
         <v>2335</v>
       </c>
       <c r="Q131" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R131" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S131" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T131" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U131" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U131" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="132" spans="1:21" x14ac:dyDescent="0.25">
@@ -43760,19 +43765,19 @@
         <v>2335</v>
       </c>
       <c r="Q132" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R132" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S132" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T132" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U132" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U132" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="133" spans="1:21" x14ac:dyDescent="0.25">
@@ -43825,16 +43830,16 @@
         <v>2335</v>
       </c>
       <c r="R133" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S133" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T133" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U133" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U133" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="134" spans="1:21" x14ac:dyDescent="0.25">
@@ -43887,19 +43892,19 @@
         <v>2323</v>
       </c>
       <c r="Q134" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R134" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S134" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T134" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U134" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U134" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="135" spans="1:21" x14ac:dyDescent="0.25">
@@ -43952,19 +43957,19 @@
         <v>2323</v>
       </c>
       <c r="Q135" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R135" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S135" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T135" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U135" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U135" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="136" spans="1:21" x14ac:dyDescent="0.25">
@@ -44017,19 +44022,19 @@
         <v>2323</v>
       </c>
       <c r="Q136" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R136" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S136" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T136" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U136" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U136" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="137" spans="1:21" x14ac:dyDescent="0.25">
@@ -44082,19 +44087,19 @@
         <v>2335</v>
       </c>
       <c r="Q137" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R137" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S137" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T137" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U137" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U137" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="138" spans="1:21" x14ac:dyDescent="0.25">
@@ -44150,16 +44155,16 @@
         <v>290</v>
       </c>
       <c r="R138" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S138" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T138" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U138" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U138" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="139" spans="1:21" x14ac:dyDescent="0.25">
@@ -44215,16 +44220,16 @@
         <v>2534</v>
       </c>
       <c r="R139" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S139" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T139" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U139" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U139" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="140" spans="1:21" x14ac:dyDescent="0.25">
@@ -44280,16 +44285,16 @@
         <v>294</v>
       </c>
       <c r="R140" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S140" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T140" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U140" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U140" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="141" spans="1:21" x14ac:dyDescent="0.25">
@@ -44345,16 +44350,16 @@
         <v>2495</v>
       </c>
       <c r="R141" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S141" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T141" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U141" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U141" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="142" spans="1:21" x14ac:dyDescent="0.25">
@@ -44407,19 +44412,19 @@
         <v>2323</v>
       </c>
       <c r="Q142" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="R142" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="S142" t="s">
-        <v>2493</v>
+        <v>2414</v>
       </c>
       <c r="T142" t="s">
-        <v>2493</v>
-      </c>
-      <c r="U142" s="1" t="s">
-        <v>2493</v>
+        <v>2414</v>
+      </c>
+      <c r="U142" t="s">
+        <v>2414</v>
       </c>
     </row>
     <row r="143" spans="1:21" x14ac:dyDescent="0.25">
@@ -45809,13 +45814,14 @@
       <c r="U604" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U1" xr:uid="{B785887B-576B-4D81-AE70-D107EA8277F5}"/>
+  <autoFilter ref="A1:U1" xr:uid="{B785887B-576B-4D81-AE70-D107EA8277F5}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U142">
+      <sortCondition ref="A1"/>
+    </sortState>
+  </autoFilter>
   <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <ignoredErrors>
-    <ignoredError sqref="D6" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 

</xml_diff>